<commit_message>
Ładowanie US już działa
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/Updates/UliceOsobowe.xlsx
+++ b/TerytLoad/AppData/Updates/UliceOsobowe.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\TerytLoad\TerytLoad\AppData\Updates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{640B4B7C-6BB6-40EC-9156-A768D43D4F8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60048219-2DC2-4D28-A68D-EF92B5ABD2D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UliceOsobowe" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21494" uniqueCount="8211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21499" uniqueCount="8214">
   <si>
     <t>skwer</t>
   </si>
@@ -24666,6 +24666,15 @@
   </si>
   <si>
     <t>Mateusza Apostoła i Ewangelisty</t>
+  </si>
+  <si>
+    <t>Lindleya</t>
+  </si>
+  <si>
+    <t>Williama Lindleya</t>
+  </si>
+  <si>
+    <t>xx</t>
   </si>
 </sst>
 </file>
@@ -25545,7 +25554,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E4340"/>
+  <dimension ref="A1:E4341"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="11.7109375" customWidth="1"/>
@@ -98867,6 +98876,23 @@
         <v>5522</v>
       </c>
     </row>
+    <row r="4341" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4341" t="s">
+        <v>8213</v>
+      </c>
+      <c r="B4341" t="s">
+        <v>8213</v>
+      </c>
+      <c r="C4341" t="s">
+        <v>8211</v>
+      </c>
+      <c r="D4341" t="s">
+        <v>7613</v>
+      </c>
+      <c r="E4341" t="s">
+        <v>8212</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E4340">
     <sortCondition ref="C2:C4340"/>

</xml_diff>

<commit_message>
Poprawiony i ujednolicony match identyczny w weryfikacji ulic i ładowaniu kodów pocztowych.
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/Updates/UliceOsobowe.xlsx
+++ b/TerytLoad/AppData/Updates/UliceOsobowe.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\TerytLoad\TerytLoad\AppData\Updates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FD76972-8ADC-4806-92DF-520CD7EE0594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA948D9F-A8BE-49ED-94AD-16F001178384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21554" uniqueCount="8239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21594" uniqueCount="8247">
   <si>
     <t>skwer</t>
   </si>
@@ -24716,9 +24716,6 @@
     <t>gen. Ignacego Prądzyńskiego</t>
   </si>
   <si>
-    <t xml:space="preserve">ul. </t>
-  </si>
-  <si>
     <t>Jakubowicza</t>
   </si>
   <si>
@@ -24750,6 +24747,33 @@
   </si>
   <si>
     <t>Onufrego Zagłoby</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puszkina </t>
+  </si>
+  <si>
+    <t>Aleksandra Puszkina</t>
+  </si>
+  <si>
+    <t>Przybosia</t>
+  </si>
+  <si>
+    <t>Juliana Przybosia</t>
+  </si>
+  <si>
+    <t>Rodziewiczówny</t>
+  </si>
+  <si>
+    <t>Marii Rodziewiczówny</t>
+  </si>
+  <si>
+    <t>Chłopickiego</t>
+  </si>
+  <si>
+    <t>Józefa Chłopickiego</t>
+  </si>
+  <si>
+    <t>Tadeusza Rejtana</t>
   </si>
 </sst>
 </file>
@@ -25629,7 +25653,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E4352"/>
+  <dimension ref="A1:E4360"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="11.7109375" customWidth="1"/>
@@ -99055,27 +99079,27 @@
     </row>
     <row r="4347" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4347" t="s">
-        <v>5669</v>
+        <v>8213</v>
       </c>
       <c r="B4347" t="s">
+        <v>8213</v>
+      </c>
+      <c r="C4347" t="s">
         <v>8227</v>
-      </c>
-      <c r="C4347" t="s">
-        <v>8228</v>
       </c>
       <c r="D4347" t="s">
         <v>3632</v>
       </c>
       <c r="E4347" t="s">
-        <v>8229</v>
+        <v>8228</v>
       </c>
     </row>
     <row r="4348" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4348" t="s">
-        <v>3</v>
+        <v>8213</v>
       </c>
       <c r="B4348" t="s">
-        <v>3</v>
+        <v>8213</v>
       </c>
       <c r="C4348" t="s">
         <v>2209</v>
@@ -99089,27 +99113,27 @@
     </row>
     <row r="4349" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4349" t="s">
-        <v>5669</v>
+        <v>8213</v>
       </c>
       <c r="B4349" t="s">
-        <v>5669</v>
+        <v>8213</v>
       </c>
       <c r="C4349" t="s">
+        <v>8229</v>
+      </c>
+      <c r="D4349" t="s">
         <v>8230</v>
       </c>
-      <c r="D4349" t="s">
+      <c r="E4349" t="s">
         <v>8231</v>
-      </c>
-      <c r="E4349" t="s">
-        <v>8232</v>
       </c>
     </row>
     <row r="4350" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4350" t="s">
-        <v>3</v>
+        <v>8213</v>
       </c>
       <c r="B4350" t="s">
-        <v>3</v>
+        <v>8213</v>
       </c>
       <c r="C4350" t="s">
         <v>5322</v>
@@ -99123,36 +99147,172 @@
     </row>
     <row r="4351" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4351" t="s">
-        <v>5669</v>
+        <v>8213</v>
       </c>
       <c r="B4351" t="s">
-        <v>8227</v>
+        <v>8213</v>
       </c>
       <c r="C4351" t="s">
+        <v>8232</v>
+      </c>
+      <c r="D4351" t="s">
         <v>8233</v>
       </c>
-      <c r="D4351" t="s">
+      <c r="E4351" t="s">
         <v>8234</v>
-      </c>
-      <c r="E4351" t="s">
-        <v>8235</v>
       </c>
     </row>
     <row r="4352" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4352" t="s">
-        <v>5669</v>
+        <v>8213</v>
       </c>
       <c r="B4352" t="s">
-        <v>5669</v>
+        <v>8213</v>
       </c>
       <c r="C4352" t="s">
+        <v>8235</v>
+      </c>
+      <c r="D4352" t="s">
         <v>8236</v>
       </c>
-      <c r="D4352" t="s">
+      <c r="E4352" t="s">
         <v>8237</v>
       </c>
-      <c r="E4352" t="s">
+    </row>
+    <row r="4353" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4353" t="s">
+        <v>8213</v>
+      </c>
+      <c r="B4353" t="s">
+        <v>8213</v>
+      </c>
+      <c r="C4353" t="s">
         <v>8238</v>
+      </c>
+      <c r="D4353" t="s">
+        <v>365</v>
+      </c>
+      <c r="E4353" t="s">
+        <v>8239</v>
+      </c>
+    </row>
+    <row r="4354" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4354" t="s">
+        <v>8213</v>
+      </c>
+      <c r="B4354" t="s">
+        <v>8213</v>
+      </c>
+      <c r="C4354" t="s">
+        <v>8240</v>
+      </c>
+      <c r="D4354" t="s">
+        <v>653</v>
+      </c>
+      <c r="E4354" t="s">
+        <v>8241</v>
+      </c>
+    </row>
+    <row r="4355" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4355" t="s">
+        <v>8213</v>
+      </c>
+      <c r="B4355" t="s">
+        <v>8213</v>
+      </c>
+      <c r="C4355" t="s">
+        <v>8242</v>
+      </c>
+      <c r="D4355" t="s">
+        <v>3673</v>
+      </c>
+      <c r="E4355" t="s">
+        <v>8243</v>
+      </c>
+    </row>
+    <row r="4356" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4356" t="s">
+        <v>8213</v>
+      </c>
+      <c r="B4356" t="s">
+        <v>8213</v>
+      </c>
+      <c r="C4356" t="s">
+        <v>1708</v>
+      </c>
+      <c r="D4356" t="s">
+        <v>225</v>
+      </c>
+      <c r="E4356" t="s">
+        <v>1707</v>
+      </c>
+    </row>
+    <row r="4357" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4357" t="s">
+        <v>8213</v>
+      </c>
+      <c r="B4357" t="s">
+        <v>8213</v>
+      </c>
+      <c r="C4357" t="s">
+        <v>2040</v>
+      </c>
+      <c r="D4357" t="s">
+        <v>181</v>
+      </c>
+      <c r="E4357" t="s">
+        <v>6512</v>
+      </c>
+    </row>
+    <row r="4358" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4358" t="s">
+        <v>8213</v>
+      </c>
+      <c r="B4358" t="s">
+        <v>8213</v>
+      </c>
+      <c r="C4358" t="s">
+        <v>8244</v>
+      </c>
+      <c r="D4358" t="s">
+        <v>262</v>
+      </c>
+      <c r="E4358" t="s">
+        <v>8245</v>
+      </c>
+    </row>
+    <row r="4359" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4359" t="s">
+        <v>8213</v>
+      </c>
+      <c r="B4359" t="s">
+        <v>8213</v>
+      </c>
+      <c r="C4359" t="s">
+        <v>4056</v>
+      </c>
+      <c r="D4359" t="s">
+        <v>492</v>
+      </c>
+      <c r="E4359" t="s">
+        <v>8246</v>
+      </c>
+    </row>
+    <row r="4360" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4360" t="s">
+        <v>8213</v>
+      </c>
+      <c r="B4360" t="s">
+        <v>8213</v>
+      </c>
+      <c r="C4360" t="s">
+        <v>463</v>
+      </c>
+      <c r="D4360" t="s">
+        <v>5202</v>
+      </c>
+      <c r="E4360" t="s">
+        <v>5905</v>
       </c>
     </row>
   </sheetData>

</xml_diff>